<commit_message>
Update Birthday Memo data
</commit_message>
<xml_diff>
--- a/Birthdays.xlsx
+++ b/Birthdays.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="36.6328125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -1363,6 +1363,28 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>8/8/2026 17:31:04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>4/16/1988</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Chetan</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1/31/2015</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
cLEAN test data and sync birthday state
</commit_message>
<xml_diff>
--- a/Birthdays.xlsx
+++ b/Birthdays.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="19200" windowHeight="6800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,43 +12,387 @@
     <sheet name="Duplicate_Check" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Birthday_View'!$A$1:$E$58</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Birthday_Calendar'!$A$1:$E$58</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Duplicate_Check'!$A$1:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Birthday_View'!$A$1:$E$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Birthday_Calendar'!$A$1:$E$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Duplicate_Check'!$A$1:$E$4</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <charset val="134"/>
       <b val="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -56,24 +400,311 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -442,7 +1073,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -452,12 +1082,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:D59"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col width="17.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="19.81640625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="36.6328125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="17.1818181818182" customWidth="1" min="1" max="1"/>
+    <col width="19.8181818181818" customWidth="1" min="2" max="2"/>
+    <col width="36.6363636363636" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,1190 +1183,1163 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7/18/2026 10:58:08</t>
+          <t>7/18/2026 10:40:51</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1/11/1988</t>
+          <t>12/28/1986</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Manisha Singhal</t>
+          <t xml:space="preserve">Prasanjeet </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7/18/2026 11:26:16</t>
+          <t>7/18/2026 10:58:08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10/28/1988</t>
+          <t>1/11/1988</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bhumika chaudhary</t>
+          <t>Manisha Singhal</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7/18/2026 11:41:18</t>
+          <t>7/18/2026 11:26:16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1/8/1988</t>
+          <t>10/28/1988</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nitin chawla</t>
+          <t>Bhumika chaudhary</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7/18/2026 11:45:55</t>
+          <t>7/18/2026 11:41:18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8/25/1987</t>
+          <t>1/8/1988</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lavi Aggarwal </t>
+          <t>Nitin chawla</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7/18/2026 12:08:57</t>
+          <t>7/18/2026 11:45:55</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8/5/1988</t>
+          <t>8/25/1987</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Swati Tyagi </t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>11/27/2009</t>
+          <t xml:space="preserve">Lavi Aggarwal </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7/18/2026 12:11:49</t>
+          <t>7/18/2026 12:08:57</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/4/2026</t>
+          <t>8/5/1988</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ishan Bhardwaj</t>
+          <t xml:space="preserve">Swati Tyagi </t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>11/27/2009</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7/18/2026 12:42:43</t>
+          <t>7/18/2026 12:11:49</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/18/1987</t>
+          <t>12/4/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SEERAT KAUR (FORMERLY SUMIT KAPOOR)</t>
+          <t>Ishan Bhardwaj</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11/4/2012</t>
+          <t>10/31/2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7/18/2026 13:05:39</t>
+          <t>7/18/2026 12:42:43</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5/17/2026</t>
+          <t>12/18/1987</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MUKUL</t>
+          <t>SEERAT KAUR (FORMERLY SUMIT KAPOOR)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12/8/2026</t>
+          <t>11/4/2012</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7/18/2026 13:11:40</t>
+          <t>7/18/2026 13:05:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12/28/1986</t>
+          <t>5/17/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prasanjeet </t>
+          <t>MUKUL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7/10/2013</t>
+          <t>12/8/2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>7/18/2026 16:15:56</t>
+          <t>7/18/2026 13:11:40</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7/20/1987</t>
+          <t>12/28/1986</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pallavi Tomar</t>
+          <t xml:space="preserve">Prasanjeet </t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2/20/2009</t>
+          <t>7/10/2013</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>7/18/2026 18:15:22</t>
+          <t>7/18/2026 13:31:29</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1/26/1987</t>
+          <t>10/5/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Rajan</t>
+          <t xml:space="preserve">Jaspreet </t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11/20/2022</t>
+          <t>4/5/2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>7/18/2026 18:24:05</t>
+          <t>7/18/2026 16:15:56</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10/30/1987</t>
+          <t>7/20/1987</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nimesh</t>
+          <t>Pallavi Tomar</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>11/28/2013</t>
+          <t>2/20/2009</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>7/18/2026 22:58:38</t>
+          <t>7/18/2026 18:15:22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11/28/1987</t>
+          <t>1/26/1987</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SUMIT CHHABRA</t>
+          <t>Rajan</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4/19/2015</t>
+          <t>11/20/2022</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>7/19/2026 7:35:25</t>
+          <t>7/18/2026 18:24:05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2/17/1988</t>
+          <t>10/30/1987</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shringika </t>
+          <t>Nimesh</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>12/9/2016</t>
+          <t>11/28/2013</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7/19/2026 9:38:34</t>
+          <t>7/18/2026 22:58:38</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2/22/2026</t>
+          <t>11/28/1987</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Yadu Nagar</t>
+          <t>SUMIT CHHABRA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1/26/2026</t>
+          <t>4/19/2015</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7/19/2026 10:23:13</t>
+          <t>7/19/2026 7:35:25</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>7/10/1987</t>
+          <t>2/17/1988</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Kavita Babbar</t>
+          <t xml:space="preserve">Shringika </t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1/29/2016</t>
+          <t>12/9/2016</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7/20/2026 8:35:57</t>
+          <t>7/19/2026 9:38:34</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/18/1987</t>
+          <t>2/22/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Priyanka Verma </t>
+          <t>Yadu Nagar</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>6/7/2010</t>
+          <t>1/26/2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7/20/2026 8:39:31</t>
+          <t>7/19/2026 10:23:13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1/29/1988</t>
+          <t>7/10/1987</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shruti kaushal </t>
+          <t>Kavita Babbar</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>12/6/2014</t>
+          <t>1/29/2016</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7/20/2026 9:17:29</t>
+          <t>7/20/2026 8:35:57</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>9/17/1988</t>
+          <t>10/18/1987</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sakshi Goel Agarwal</t>
+          <t xml:space="preserve">Priyanka Verma </t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>12/3/2014</t>
+          <t>6/7/2010</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7/20/2026 9:34:23</t>
+          <t>7/20/2026 8:39:31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/1/1987</t>
+          <t>1/29/1988</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Swati Aggarwal(Bishnoi)🙂</t>
+          <t xml:space="preserve">Shruti kaushal </t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1/20/2010</t>
+          <t>12/6/2014</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7/20/2026 10:37:24</t>
+          <t>7/20/2026 9:17:29</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1/22/1987</t>
+          <t>9/17/1988</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Abhishek Goel</t>
+          <t>Sakshi Goel Agarwal</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2/15/2014</t>
+          <t>12/3/2014</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7/20/2026 11:10:45</t>
+          <t>7/20/2026 9:34:23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4/11/1987</t>
+          <t>10/1/1987</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mohit sharma</t>
+          <t>Swati Aggarwal(Bishnoi)🙂</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1/23/2013</t>
+          <t>1/20/2010</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7/20/2026 11:12:35</t>
+          <t>7/20/2026 10:37:24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>9/21/2026</t>
+          <t>1/22/1987</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Richa Sharma </t>
+          <t>Abhishek Goel</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1/18/2026</t>
+          <t>2/15/2014</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7/20/2026 14:58:09</t>
+          <t>7/20/2026 11:10:45</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>7/8/2026</t>
+          <t>4/11/1987</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ashish tyagi </t>
+          <t>Mohit sharma</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>11/25/2020</t>
+          <t>1/23/2013</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7/20/2026 16:24:06</t>
+          <t>7/20/2026 11:12:35</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>8/4/1987</t>
+          <t>9/21/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Shatakshi Verma</t>
+          <t xml:space="preserve">Richa Sharma </t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1/19/2013</t>
+          <t>1/18/2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7/21/2026 10:13:47</t>
+          <t>7/20/2026 14:58:09</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>7/28/1988</t>
+          <t>7/8/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Jatin</t>
+          <t xml:space="preserve">Ashish tyagi </t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5/9/2015</t>
+          <t>11/25/2020</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7/21/2026 20:51:57</t>
+          <t>7/20/2026 16:24:06</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>8/19/0087</t>
+          <t>8/4/1987</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Vibhor Agarwal</t>
+          <t>Shatakshi Verma</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>11/24/0012</t>
+          <t>1/19/2013</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>8/7/2026 7:03:08</t>
+          <t>7/21/2026 10:13:47</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>8/7/1988</t>
+          <t>7/28/1988</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Harsh Dutt</t>
+          <t>Jatin</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>7/27/2026</t>
+          <t>5/9/2015</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>8/7/2026 7:03:46</t>
+          <t>7/21/2026 20:51:57</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>8/7/1988</t>
+          <t>8/19/0087</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Dhirendra</t>
+          <t>Vibhor Agarwal</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>8/7/2026</t>
+          <t>11/24/0012</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>8/7/2026 7:04:17</t>
+          <t>8/7/2026 7:03:08</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>8/8/1988</t>
+          <t>8/7/1988</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Rohit Pradhan</t>
+          <t>Harsh Dutt</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>8/4/2026</t>
+          <t>7/27/2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>8/7/2026 8:05:15</t>
+          <t>8/7/2026 7:03:46</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>7/9/1987</t>
+          <t>8/7/1988</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ayush manglik</t>
+          <t>Dhirendra</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>12/9/2016</t>
+          <t>8/7/2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8/7/2026 8:53:13</t>
+          <t>8/7/2026 7:04:17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>8/4/1987</t>
+          <t>8/8/1988</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Shatakshi Verma</t>
+          <t>Rohit Pradhan</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1/19/2013</t>
+          <t>8/4/2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>8/7/2026 12:51:53</t>
+          <t>8/7/2026 8:05:15</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>12/29/1986</t>
+          <t>7/9/1987</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ashu Garg</t>
+          <t>Ayush manglik</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>4/17/2016</t>
+          <t>12/9/2016</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>8/8/2026 15:35:52</t>
+          <t>8/7/2026 8:53:13</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1/7/1988</t>
+          <t>8/4/1987</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Vikrant</t>
+          <t>Shatakshi Verma</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>8/8/2026</t>
+          <t>1/19/2013</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8/8/2026 16:22:47</t>
+          <t>8/7/2026 12:51:53</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/13/1986</t>
+          <t>12/29/1986</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shobhit kaushik </t>
+          <t>Ashu Garg</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>11/24/2016</t>
+          <t>4/17/2016</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8/8/2026 17:02:42</t>
+          <t>8/8/2026 15:35:52</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>12/10/1987</t>
+          <t>1/7/1988</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Shashank Chaudhary</t>
+          <t>Vikrant</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>4/17/2016</t>
+          <t>8/8/2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>8/8/2026 17:02:56</t>
+          <t>8/8/2026 16:22:47</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>5/17/1988</t>
+          <t>11/13/1986</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>mukul</t>
+          <t xml:space="preserve">Shobhit kaushik </t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>12/8/2013</t>
+          <t>11/24/2016</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>8/8/2026 17:31:04</t>
+          <t>8/8/2026 16:24:08</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>4/16/1988</t>
+          <t>7/21/1988</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Chetan</t>
+          <t>Rekha Lakchaura</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1/31/2015</t>
+          <t>8/8/2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>8/8/2026 19:03:11</t>
+          <t>8/8/2026 17:02:42</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>8/31/1987</t>
+          <t>12/10/1987</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ajeet Singh</t>
+          <t>Shashank Chaudhary</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>1/16/2017</t>
+          <t>4/17/2016</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>8/8/2026 19:10:07</t>
+          <t>8/8/2026 17:02:56</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>10/1/1987</t>
+          <t>5/17/1988</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Swati Bishnoi</t>
+          <t>mukul</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>1/20/2010</t>
+          <t>12/8/2013</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>8/8/2026 19:13:41</t>
+          <t>8/8/2026 17:31:04</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>5/7/1988</t>
+          <t>4/16/1988</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mayank Gambhir</t>
+          <t>Chetan</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>8/8/1837</t>
+          <t>1/31/2015</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>8/8/2026 19:39:21</t>
+          <t>8/8/2026 19:03:11</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>7/21/2026</t>
+          <t>8/31/1987</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Rekha</t>
+          <t>Ajeet Singh</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4/26/2014</t>
+          <t>1/16/2017</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>8/9/2026 10:26:31</t>
+          <t>8/8/2026 19:10:07</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1/22/2026</t>
+          <t>10/1/1987</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Shrey dhingra</t>
+          <t>Swati Bishnoi</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2/19/2026</t>
+          <t>1/20/2010</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>8/9/2026 15:46:07</t>
+          <t>8/8/2026 19:13:41</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1/5/1988</t>
+          <t>5/7/1988</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sanjeev kumar</t>
+          <t>Mayank Gambhir</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2/19/2018</t>
+          <t>8/8/1837</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>8/13/2026 8:28:48</t>
+          <t>8/8/2026 19:23:01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>7/8/1988</t>
+          <t>8/5/1988</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Ashish tyagi</t>
+          <t>Xyz</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>11/25/2020</t>
+          <t>8/8/2026</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>8/13/2026 9:17:34</t>
+          <t>8/8/2026 19:39:21</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>12/4/1986</t>
+          <t>7/21/2026</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ishan Bhardwaj</t>
+          <t>Rekha</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10/31/2017</t>
+          <t>4/26/2014</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>8/13/2026 9:44:22</t>
+          <t>8/9/2026 10:26:31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>10/5/1987</t>
+          <t>1/22/2026</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Jaspreet Sethi</t>
+          <t>Shrey dhingra</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>4/5/2015</t>
+          <t>2/19/2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>8/14/2026 20:28:49</t>
+          <t>8/9/2026 15:46:07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>12/7/1988</t>
+          <t>1/5/1988</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kriti Sharma </t>
+          <t>sanjeev kumar</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2/15/2014</t>
+          <t>2/19/2018</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>8/14/2026 22:28:29</t>
+          <t>8/13/2026 8:28:48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>4/16/1987</t>
+          <t>7/8/1988</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Tanuj Sablok</t>
+          <t>Ashish tyagi</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>8/14/2026</t>
+          <t>11/25/2020</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>8/14/2026 22:56:43</t>
+          <t>8/13/2026 9:17:34</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>8/14/1988</t>
+          <t>12/4/1986</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Vivek Ahlawat</t>
+          <t>Ishan Bhardwaj</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>8/14/2026</t>
+          <t>10/31/2017</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>8/16/2026 12:38:07</t>
+          <t>8/13/2026 9:44:22</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>8/2/1988</t>
+          <t>10/5/1987</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Test Birthday</t>
+          <t>Jaspreet Sethi</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>8/16/2026</t>
+          <t>4/5/2015</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>8/16/2026 12:45:07</t>
+          <t>8/14/2026 20:28:49</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>8/6/1983</t>
+          <t>12/7/1988</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Testing </t>
+          <t xml:space="preserve">Kriti Sharma </t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>8/16/2026</t>
+          <t>2/15/2014</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>8/17/2026 5:47:53</t>
+          <t>8/14/2026 22:28:29</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>8/1/1990</t>
+          <t>4/16/1987</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Testing entity</t>
+          <t>Tanuj Sablok</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>8/19/2026</t>
+          <t>8/14/2026</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>8/17/2026 13:06:48</t>
+          <t>8/14/2026 22:56:43</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>8/17/1988</t>
+          <t>8/14/1988</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Testing entity</t>
+          <t>Vivek Ahlawat</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>8/17/2000</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>8/17/2026 22:06:26</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>12/24/2010</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>testing</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>8/17/2026</t>
+          <t>8/14/2026</t>
         </is>
       </c>
     </row>
@@ -1751,7 +2354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1762,27 +2365,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Birthday</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Birthday_Current</t>
         </is>
@@ -2320,12 +2923,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Jatin</t>
+          <t>Rekha Lakchaura</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>7/28/1988</t>
+          <t>7/21/1988</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2334,7 +2937,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -2343,21 +2946,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Testing entity</t>
+          <t>Jatin</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>8/1/1990</t>
+          <t>7/28/1988</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>July</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -2366,12 +2969,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Test Birthday</t>
+          <t>Shatakshi Verma</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>8/2/1988</t>
+          <t>8/4/1987</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2380,7 +2983,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -2389,12 +2992,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Shatakshi Verma</t>
+          <t>Swati Tyagi</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>8/4/1987</t>
+          <t>8/5/1988</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2403,7 +3006,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -2412,7 +3015,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Swati Tyagi</t>
+          <t>Xyz</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2435,12 +3038,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Dhirendra</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>8/6/1983</t>
+          <t>8/7/1988</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2449,7 +3052,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -2458,7 +3061,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dhirendra</t>
+          <t>Harsh Dutt</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2481,12 +3084,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Harsh Dutt</t>
+          <t>Rohit Pradhan</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>8/7/1988</t>
+          <t>8/8/1988</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2495,7 +3098,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -2504,12 +3107,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Rohit Pradhan</t>
+          <t>Vivek Ahlawat</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>8/8/1988</t>
+          <t>8/14/1988</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2518,7 +3121,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -2527,12 +3130,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Vivek Ahlawat</t>
+          <t>Vibhor Agarwal</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>8/14/1988</t>
+          <t>8/19/0087</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2541,7 +3144,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -2550,12 +3153,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Testing entity</t>
+          <t>Lavi Aggarwal</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>8/17/1988</t>
+          <t>8/25/1987</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2564,21 +3167,21 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Vibhor Agarwal</t>
+          <t>Ajeet Singh</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>8/19/0087</t>
+          <t>8/31/1987</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2587,7 +3190,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -2596,21 +3199,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lavi Aggarwal</t>
+          <t>Sakshi Goel Agarwal</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>8/25/1987</t>
+          <t>9/17/1988</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -2619,21 +3222,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ajeet Singh</t>
+          <t>Richa Sharma</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>8/31/1987</t>
+          <t>9/21/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -2642,21 +3245,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sakshi Goel Agarwal</t>
+          <t>Swati Aggarwal(Bishnoi)🙂</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>9/17/1988</t>
+          <t>10/1/1987</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -2665,21 +3268,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Richa Sharma</t>
+          <t>Jaspreet</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>9/21/2026</t>
+          <t>10/5/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -2688,12 +3291,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Swati Aggarwal(Bishnoi)🙂</t>
+          <t>Jaspreet Sethi</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10/1/1987</t>
+          <t>10/5/1987</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2702,7 +3305,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -2711,12 +3314,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jaspreet Sethi</t>
+          <t>Priyanka Verma</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10/5/1987</t>
+          <t>10/18/1987</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2725,7 +3328,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -2734,12 +3337,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Priyanka Verma</t>
+          <t>Bhumika chaudhary</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10/18/1987</t>
+          <t>10/28/1988</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2748,7 +3351,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -2757,12 +3360,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Bhumika chaudhary</t>
+          <t>Nimesh</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10/28/1988</t>
+          <t>10/30/1987</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2771,7 +3374,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -2780,21 +3383,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Nimesh</t>
+          <t>Shobhit kaushik</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>10/30/1987</t>
+          <t>11/13/1986</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -2803,12 +3406,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Shobhit kaushik</t>
+          <t>Pratyaksh Tomar</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/13/1986</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2817,7 +3420,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -2826,12 +3429,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pratyaksh Tomar</t>
+          <t>SUMIT CHHABRA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/28/1987</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2849,21 +3452,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SUMIT CHHABRA</t>
+          <t>Ishan Bhardwaj</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>11/28/1987</t>
+          <t>12/4/2026</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>November</t>
+          <t>December</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -2877,7 +3480,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12/4/2026</t>
+          <t>12/4/1986</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2895,12 +3498,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ishan Bhardwaj</t>
+          <t>Isha shukla</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>12/4/1986</t>
+          <t>12/6/0086</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2909,7 +3512,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -2918,12 +3521,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Isha shukla</t>
+          <t>Kriti Sharma</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>12/6/0086</t>
+          <t>12/7/1988</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2932,7 +3535,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -2941,12 +3544,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Kriti Sharma</t>
+          <t>Shashank Chaudhary</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>12/7/1988</t>
+          <t>12/10/1987</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2955,7 +3558,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -2964,12 +3567,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Shashank Chaudhary</t>
+          <t>Gopal Verma</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>12/10/1987</t>
+          <t>12/17/1987</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2978,7 +3581,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -2987,12 +3590,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Gopal Verma</t>
+          <t>SEERAT KAUR (FORMERLY SUMIT KAPOOR)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>12/17/1987</t>
+          <t>12/18/1987</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3001,7 +3604,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -3010,12 +3613,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SEERAT KAUR (FORMERLY SUMIT KAPOOR)</t>
+          <t>Prasanjeet</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>12/18/1987</t>
+          <t>12/28/1986</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3024,7 +3627,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -3033,12 +3636,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>testing</t>
+          <t>Ashu Garg</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>12/24/2010</t>
+          <t>12/29/1986</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3047,61 +3650,15 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Prasanjeet</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>12/28/1986</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>December</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>28</v>
-      </c>
-      <c r="E57" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Ashu Garg</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>12/29/1986</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>December</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>29</v>
-      </c>
-      <c r="E58" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E58"/>
-  <conditionalFormatting sqref="A2:E58">
+  <autoFilter ref="A1:E56"/>
+  <conditionalFormatting sqref="A2:E56">
     <cfRule type="expression" priority="1" dxfId="1">
       <formula>$E2=TRUE</formula>
     </cfRule>
@@ -3116,7 +3673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3127,27 +3684,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Birthday</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Birthday_Current</t>
         </is>
@@ -3689,16 +4246,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Jatin</t>
+          <t>Rekha Lakchaura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>7/28/1988</t>
+          <t>7/21/1988</t>
         </is>
       </c>
       <c r="E25" t="b">
@@ -3708,20 +4265,20 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>July</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Testing entity</t>
+          <t>Jatin</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>8/1/1990</t>
+          <t>7/28/1988</t>
         </is>
       </c>
       <c r="E26" t="b">
@@ -3735,16 +4292,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Test Birthday</t>
+          <t>Shatakshi Verma</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>8/2/1988</t>
+          <t>8/4/1987</t>
         </is>
       </c>
       <c r="E27" t="b">
@@ -3758,16 +4315,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Shatakshi Verma</t>
+          <t>Swati Tyagi</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>8/4/1987</t>
+          <t>8/5/1988</t>
         </is>
       </c>
       <c r="E28" t="b">
@@ -3785,7 +4342,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Swati Tyagi</t>
+          <t>Xyz</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3804,16 +4361,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Dhirendra</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>8/6/1983</t>
+          <t>8/7/1988</t>
         </is>
       </c>
       <c r="E30" t="b">
@@ -3831,7 +4388,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dhirendra</t>
+          <t>Harsh Dutt</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3850,16 +4407,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Harsh Dutt</t>
+          <t>Rohit Pradhan</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>8/7/1988</t>
+          <t>8/8/1988</t>
         </is>
       </c>
       <c r="E32" t="b">
@@ -3873,16 +4430,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Rohit Pradhan</t>
+          <t>Vivek Ahlawat</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>8/8/1988</t>
+          <t>8/14/1988</t>
         </is>
       </c>
       <c r="E33" t="b">
@@ -3896,16 +4453,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Vivek Ahlawat</t>
+          <t>Vibhor Agarwal</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>8/14/1988</t>
+          <t>8/19/0087</t>
         </is>
       </c>
       <c r="E34" t="b">
@@ -3919,20 +4476,20 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Testing entity</t>
+          <t>Lavi Aggarwal</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>8/17/1988</t>
+          <t>8/25/1987</t>
         </is>
       </c>
       <c r="E35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -3942,16 +4499,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Vibhor Agarwal</t>
+          <t>Ajeet Singh</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>8/19/0087</t>
+          <t>8/31/1987</t>
         </is>
       </c>
       <c r="E36" t="b">
@@ -3961,20 +4518,20 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lavi Aggarwal</t>
+          <t>Sakshi Goel Agarwal</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>8/25/1987</t>
+          <t>9/17/1988</t>
         </is>
       </c>
       <c r="E37" t="b">
@@ -3984,20 +4541,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>September</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ajeet Singh</t>
+          <t>Richa Sharma</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>8/31/1987</t>
+          <t>9/21/2026</t>
         </is>
       </c>
       <c r="E38" t="b">
@@ -4007,20 +4564,20 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Sakshi Goel Agarwal</t>
+          <t>Swati Aggarwal(Bishnoi)🙂</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>9/17/1988</t>
+          <t>10/1/1987</t>
         </is>
       </c>
       <c r="E39" t="b">
@@ -4030,20 +4587,20 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>October</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Richa Sharma</t>
+          <t>Jaspreet</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9/21/2026</t>
+          <t>10/5/2026</t>
         </is>
       </c>
       <c r="E40" t="b">
@@ -4057,16 +4614,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Swati Aggarwal(Bishnoi)🙂</t>
+          <t>Jaspreet Sethi</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10/1/1987</t>
+          <t>10/5/1987</t>
         </is>
       </c>
       <c r="E41" t="b">
@@ -4080,16 +4637,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Jaspreet Sethi</t>
+          <t>Priyanka Verma</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10/5/1987</t>
+          <t>10/18/1987</t>
         </is>
       </c>
       <c r="E42" t="b">
@@ -4103,16 +4660,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Priyanka Verma</t>
+          <t>Bhumika chaudhary</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10/18/1987</t>
+          <t>10/28/1988</t>
         </is>
       </c>
       <c r="E43" t="b">
@@ -4126,16 +4683,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bhumika chaudhary</t>
+          <t>Nimesh</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10/28/1988</t>
+          <t>10/30/1987</t>
         </is>
       </c>
       <c r="E44" t="b">
@@ -4145,20 +4702,20 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>November</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Nimesh</t>
+          <t>Shobhit kaushik</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10/30/1987</t>
+          <t>11/13/1986</t>
         </is>
       </c>
       <c r="E45" t="b">
@@ -4172,16 +4729,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Shobhit kaushik</t>
+          <t>Pratyaksh Tomar</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>11/13/1986</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="E46" t="b">
@@ -4199,12 +4756,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Pratyaksh Tomar</t>
+          <t>SUMIT CHHABRA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/28/1987</t>
         </is>
       </c>
       <c r="E47" t="b">
@@ -4214,20 +4771,20 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>November</t>
+          <t>December</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SUMIT CHHABRA</t>
+          <t>Ishan Bhardwaj</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>11/28/1987</t>
+          <t>12/4/2026</t>
         </is>
       </c>
       <c r="E48" t="b">
@@ -4250,7 +4807,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>12/4/2026</t>
+          <t>12/4/1986</t>
         </is>
       </c>
       <c r="E49" t="b">
@@ -4264,16 +4821,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Ishan Bhardwaj</t>
+          <t>Isha shukla</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>12/4/1986</t>
+          <t>12/6/0086</t>
         </is>
       </c>
       <c r="E50" t="b">
@@ -4287,16 +4844,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Isha shukla</t>
+          <t>Kriti Sharma</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>12/6/0086</t>
+          <t>12/7/1988</t>
         </is>
       </c>
       <c r="E51" t="b">
@@ -4310,16 +4867,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Kriti Sharma</t>
+          <t>Shashank Chaudhary</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>12/7/1988</t>
+          <t>12/10/1987</t>
         </is>
       </c>
       <c r="E52" t="b">
@@ -4333,16 +4890,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Shashank Chaudhary</t>
+          <t>Gopal Verma</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>12/10/1987</t>
+          <t>12/17/1987</t>
         </is>
       </c>
       <c r="E53" t="b">
@@ -4356,16 +4913,16 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Gopal Verma</t>
+          <t>SEERAT KAUR (FORMERLY SUMIT KAPOOR)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>12/17/1987</t>
+          <t>12/18/1987</t>
         </is>
       </c>
       <c r="E54" t="b">
@@ -4379,16 +4936,16 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SEERAT KAUR (FORMERLY SUMIT KAPOOR)</t>
+          <t>Prasanjeet</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>12/18/1987</t>
+          <t>12/28/1986</t>
         </is>
       </c>
       <c r="E55" t="b">
@@ -4402,71 +4959,25 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>testing</t>
+          <t>Ashu Garg</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>12/24/2010</t>
+          <t>12/29/1986</t>
         </is>
       </c>
       <c r="E56" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>December</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>28</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Prasanjeet</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>12/28/1986</t>
-        </is>
-      </c>
-      <c r="E57" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>December</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>29</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Ashu Garg</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>12/29/1986</t>
-        </is>
-      </c>
-      <c r="E58" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E58"/>
-  <conditionalFormatting sqref="A2:E58">
+  <autoFilter ref="A1:E56"/>
+  <conditionalFormatting sqref="A2:E56">
     <cfRule type="expression" priority="1" dxfId="1">
       <formula>$E2=TRUE</formula>
     </cfRule>
@@ -4481,7 +4992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4492,27 +5003,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Kept_Name</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Kept_Birthday</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Ignored_Name</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Ignored_Birthday</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
@@ -4521,59 +5032,86 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Swati Aggarwal(Bishnoi)🙂</t>
+          <t>Prasanjeet</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10/1/1987</t>
+          <t>12/28/1986</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Swati Bishnoi</t>
+          <t>Prasanjeet</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10/1/1987</t>
+          <t>12/28/1986</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Same first name and DOB; multiple full-name entries</t>
+          <t>Same first name and DOB; duplicate first-name entry</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Swati Aggarwal(Bishnoi)🙂</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10/1/1987</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Swati Bishnoi</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10/1/1987</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Same first name and DOB; multiple full-name entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Shatakshi Verma</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>8/4/1987</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Shatakshi Verma</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>8/4/1987</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Same first name and DOB; multiple full-name entries</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E3"/>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>